<commit_message>
add intl urls for Shanghai Conservatory & CDUTCM
</commit_message>
<xml_diff>
--- a/dataset/全国重点院校/全国高校汇总表.xlsx
+++ b/dataset/全国重点院校/全国高校汇总表.xlsx
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11465" uniqueCount="1665">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11465" uniqueCount="1670">
   <si>
     <t>全国高校汇总表（就业/研究生/国际处 渠道 + 软科排名 + 二维码，按985-211-双一流-双非排列）</t>
   </si>
@@ -4325,12 +4325,15 @@
     <t>第二军医大学</t>
   </si>
   <si>
+    <t>军队院校，国际处信息不公开</t>
+  </si>
+  <si>
+    <t>第四军医大学</t>
+  </si>
+  <si>
     <t>官网未知</t>
   </si>
   <si>
-    <t>第四军医大学</t>
-  </si>
-  <si>
     <t>苏州大学</t>
   </si>
   <si>
@@ -4610,6 +4613,9 @@
     <t>上海音乐学院</t>
   </si>
   <si>
+    <t>https://www.shcmusic.edu.cn/1449/list.htm</t>
+  </si>
+  <si>
     <t>中国人民公安大学</t>
   </si>
   <si>
@@ -4869,6 +4875,15 @@
   </si>
   <si>
     <t>82713803; 82717572; 82716812</t>
+  </si>
+  <si>
+    <t>https://zyd.cdutcm.edu.cn/gjjyxy</t>
+  </si>
+  <si>
+    <t>info@cdutcm.edu.cn; IEC.GATQ@cdutcm.edu.cn; training@cdutcm.edu.cn</t>
+  </si>
+  <si>
+    <t>028-87784542; 028-87717870; 028-82682484</t>
   </si>
   <si>
     <t>成都理工大学</t>
@@ -21009,7 +21024,7 @@
         <v>29</v>
       </c>
       <c r="T247" s="6" t="s">
-        <v>1426</v>
+        <v>1428</v>
       </c>
     </row>
     <row r="248" spans="1:20">
@@ -21020,7 +21035,7 @@
         <v>962</v>
       </c>
       <c r="C248" s="6" t="s">
-        <v>1428</v>
+        <v>1429</v>
       </c>
       <c r="D248" s="6" t="s">
         <v>29</v>
@@ -21035,19 +21050,19 @@
         <v>29</v>
       </c>
       <c r="H248" s="6" t="s">
-        <v>1429</v>
+        <v>1430</v>
       </c>
       <c r="I248" s="5" t="s">
         <v>29</v>
       </c>
       <c r="J248" s="6" t="s">
-        <v>1430</v>
+        <v>1431</v>
       </c>
       <c r="K248" s="6" t="s">
-        <v>1431</v>
+        <v>1432</v>
       </c>
       <c r="L248" s="6" t="s">
-        <v>1432</v>
+        <v>1433</v>
       </c>
       <c r="M248" s="5" t="s">
         <v>29</v>
@@ -21056,10 +21071,10 @@
         <v>29</v>
       </c>
       <c r="O248" s="6" t="s">
-        <v>1433</v>
+        <v>1434</v>
       </c>
       <c r="P248" s="6" t="s">
-        <v>1434</v>
+        <v>1435</v>
       </c>
       <c r="Q248" s="6" t="s">
         <v>1141</v>
@@ -21082,7 +21097,7 @@
         <v>1127</v>
       </c>
       <c r="C249" s="6" t="s">
-        <v>1435</v>
+        <v>1436</v>
       </c>
       <c r="D249" s="6" t="s">
         <v>29</v>
@@ -21097,31 +21112,31 @@
         <v>29</v>
       </c>
       <c r="H249" s="6" t="s">
-        <v>1436</v>
+        <v>1437</v>
       </c>
       <c r="I249" s="5" t="s">
         <v>29</v>
       </c>
       <c r="J249" s="6" t="s">
-        <v>1437</v>
+        <v>1438</v>
       </c>
       <c r="K249" s="6" t="s">
-        <v>1438</v>
+        <v>1439</v>
       </c>
       <c r="L249" s="6" t="s">
-        <v>1439</v>
+        <v>1440</v>
       </c>
       <c r="M249" s="6" t="s">
-        <v>1440</v>
+        <v>1441</v>
       </c>
       <c r="N249" s="6" t="s">
         <v>29</v>
       </c>
       <c r="O249" s="6" t="s">
-        <v>1441</v>
+        <v>1442</v>
       </c>
       <c r="P249" s="6" t="s">
-        <v>1442</v>
+        <v>1443</v>
       </c>
       <c r="Q249" s="5" t="s">
         <v>29</v>
@@ -21144,7 +21159,7 @@
         <v>1072</v>
       </c>
       <c r="C250" s="6" t="s">
-        <v>1443</v>
+        <v>1444</v>
       </c>
       <c r="D250" s="6" t="s">
         <v>29</v>
@@ -21159,19 +21174,19 @@
         <v>29</v>
       </c>
       <c r="H250" s="6" t="s">
-        <v>1444</v>
+        <v>1445</v>
       </c>
       <c r="I250" s="5" t="s">
         <v>29</v>
       </c>
       <c r="J250" s="6" t="s">
-        <v>1445</v>
+        <v>1446</v>
       </c>
       <c r="K250" s="6" t="s">
-        <v>1446</v>
+        <v>1447</v>
       </c>
       <c r="L250" s="6" t="s">
-        <v>1447</v>
+        <v>1448</v>
       </c>
       <c r="M250" s="5" t="s">
         <v>29</v>
@@ -21180,10 +21195,10 @@
         <v>29</v>
       </c>
       <c r="O250" s="6" t="s">
-        <v>1448</v>
+        <v>1449</v>
       </c>
       <c r="P250" s="6" t="s">
-        <v>1449</v>
+        <v>1450</v>
       </c>
       <c r="Q250" s="5" t="s">
         <v>29</v>
@@ -21206,7 +21221,7 @@
         <v>1150</v>
       </c>
       <c r="C251" s="6" t="s">
-        <v>1450</v>
+        <v>1451</v>
       </c>
       <c r="D251" s="6" t="s">
         <v>29</v>
@@ -21221,7 +21236,7 @@
         <v>29</v>
       </c>
       <c r="H251" s="6" t="s">
-        <v>1451</v>
+        <v>1452</v>
       </c>
       <c r="I251" s="5" t="s">
         <v>29</v>
@@ -21233,19 +21248,19 @@
         <v>29</v>
       </c>
       <c r="L251" s="6" t="s">
-        <v>1452</v>
+        <v>1453</v>
       </c>
       <c r="M251" s="5" t="s">
         <v>29</v>
       </c>
       <c r="N251" s="6" t="s">
-        <v>1453</v>
+        <v>1454</v>
       </c>
       <c r="O251" s="6" t="s">
         <v>29</v>
       </c>
       <c r="P251" s="6" t="s">
-        <v>1454</v>
+        <v>1455</v>
       </c>
       <c r="Q251" s="5" t="s">
         <v>29</v>
@@ -21268,7 +21283,7 @@
         <v>1072</v>
       </c>
       <c r="C252" s="6" t="s">
-        <v>1455</v>
+        <v>1456</v>
       </c>
       <c r="D252" s="6" t="s">
         <v>29</v>
@@ -21283,31 +21298,31 @@
         <v>29</v>
       </c>
       <c r="H252" s="6" t="s">
-        <v>1456</v>
+        <v>1457</v>
       </c>
       <c r="I252" s="5" t="s">
         <v>29</v>
       </c>
       <c r="J252" s="6" t="s">
-        <v>1457</v>
+        <v>1458</v>
       </c>
       <c r="K252" s="6" t="s">
-        <v>1458</v>
+        <v>1459</v>
       </c>
       <c r="L252" s="6" t="s">
-        <v>1459</v>
+        <v>1460</v>
       </c>
       <c r="M252" s="5" t="s">
         <v>29</v>
       </c>
       <c r="N252" s="6" t="s">
-        <v>1460</v>
+        <v>1461</v>
       </c>
       <c r="O252" s="6" t="s">
-        <v>1461</v>
+        <v>1462</v>
       </c>
       <c r="P252" s="6" t="s">
-        <v>1462</v>
+        <v>1463</v>
       </c>
       <c r="Q252" s="5" t="s">
         <v>29</v>
@@ -21330,7 +21345,7 @@
         <v>1127</v>
       </c>
       <c r="C253" s="6" t="s">
-        <v>1463</v>
+        <v>1464</v>
       </c>
       <c r="D253" s="6" t="s">
         <v>29</v>
@@ -21345,19 +21360,19 @@
         <v>29</v>
       </c>
       <c r="H253" s="6" t="s">
-        <v>1464</v>
+        <v>1465</v>
       </c>
       <c r="I253" s="5" t="s">
         <v>29</v>
       </c>
       <c r="J253" s="6" t="s">
-        <v>1465</v>
+        <v>1466</v>
       </c>
       <c r="K253" s="6" t="s">
-        <v>1466</v>
+        <v>1467</v>
       </c>
       <c r="L253" s="6" t="s">
-        <v>1467</v>
+        <v>1468</v>
       </c>
       <c r="M253" s="5" t="s">
         <v>29</v>
@@ -21366,10 +21381,10 @@
         <v>29</v>
       </c>
       <c r="O253" s="6" t="s">
-        <v>1468</v>
+        <v>1469</v>
       </c>
       <c r="P253" s="6" t="s">
-        <v>1469</v>
+        <v>1470</v>
       </c>
       <c r="Q253" s="5" t="s">
         <v>29</v>
@@ -21389,10 +21404,10 @@
         <v>252</v>
       </c>
       <c r="B254" s="6" t="s">
-        <v>1470</v>
+        <v>1471</v>
       </c>
       <c r="C254" s="6" t="s">
-        <v>1471</v>
+        <v>1472</v>
       </c>
       <c r="D254" s="6" t="s">
         <v>29</v>
@@ -21431,7 +21446,7 @@
         <v>29</v>
       </c>
       <c r="P254" s="6" t="s">
-        <v>1472</v>
+        <v>1473</v>
       </c>
       <c r="Q254" s="5" t="s">
         <v>29</v>
@@ -21451,10 +21466,10 @@
         <v>253</v>
       </c>
       <c r="B255" s="6" t="s">
-        <v>1473</v>
+        <v>1474</v>
       </c>
       <c r="C255" s="6" t="s">
-        <v>1474</v>
+        <v>1475</v>
       </c>
       <c r="D255" s="6" t="s">
         <v>29</v>
@@ -21469,7 +21484,7 @@
         <v>29</v>
       </c>
       <c r="H255" s="6" t="s">
-        <v>1475</v>
+        <v>1476</v>
       </c>
       <c r="I255" s="5" t="s">
         <v>29</v>
@@ -21478,10 +21493,10 @@
         <v>29</v>
       </c>
       <c r="K255" s="6" t="s">
-        <v>1476</v>
+        <v>1477</v>
       </c>
       <c r="L255" s="6" t="s">
-        <v>1477</v>
+        <v>1478</v>
       </c>
       <c r="M255" s="5" t="s">
         <v>29</v>
@@ -21493,7 +21508,7 @@
         <v>29</v>
       </c>
       <c r="P255" s="6" t="s">
-        <v>1478</v>
+        <v>1479</v>
       </c>
       <c r="Q255" s="5" t="s">
         <v>29</v>
@@ -21513,10 +21528,10 @@
         <v>254</v>
       </c>
       <c r="B256" s="6" t="s">
-        <v>1479</v>
+        <v>1480</v>
       </c>
       <c r="C256" s="6" t="s">
-        <v>1480</v>
+        <v>1481</v>
       </c>
       <c r="D256" s="6" t="s">
         <v>29</v>
@@ -21531,19 +21546,19 @@
         <v>29</v>
       </c>
       <c r="H256" s="6" t="s">
-        <v>1481</v>
+        <v>1482</v>
       </c>
       <c r="I256" s="6" t="s">
-        <v>1482</v>
+        <v>1483</v>
       </c>
       <c r="J256" s="6" t="s">
-        <v>1483</v>
+        <v>1484</v>
       </c>
       <c r="K256" s="6" t="s">
-        <v>1484</v>
+        <v>1485</v>
       </c>
       <c r="L256" s="6" t="s">
-        <v>1485</v>
+        <v>1486</v>
       </c>
       <c r="M256" s="5" t="s">
         <v>29</v>
@@ -21555,7 +21570,7 @@
         <v>29</v>
       </c>
       <c r="P256" s="6" t="s">
-        <v>1486</v>
+        <v>1487</v>
       </c>
       <c r="Q256" s="5" t="s">
         <v>29</v>
@@ -21578,7 +21593,7 @@
         <v>1127</v>
       </c>
       <c r="C257" s="6" t="s">
-        <v>1487</v>
+        <v>1488</v>
       </c>
       <c r="D257" s="6" t="s">
         <v>29</v>
@@ -21593,7 +21608,7 @@
         <v>29</v>
       </c>
       <c r="H257" s="6" t="s">
-        <v>1488</v>
+        <v>1489</v>
       </c>
       <c r="I257" s="5" t="s">
         <v>29</v>
@@ -21605,10 +21620,10 @@
         <v>29</v>
       </c>
       <c r="L257" s="6" t="s">
-        <v>1489</v>
+        <v>1490</v>
       </c>
       <c r="M257" s="6" t="s">
-        <v>1490</v>
+        <v>1491</v>
       </c>
       <c r="N257" s="6" t="s">
         <v>29</v>
@@ -21617,7 +21632,7 @@
         <v>29</v>
       </c>
       <c r="P257" s="6" t="s">
-        <v>1491</v>
+        <v>1492</v>
       </c>
       <c r="Q257" s="5" t="s">
         <v>29</v>
@@ -21640,7 +21655,7 @@
         <v>1127</v>
       </c>
       <c r="C258" s="6" t="s">
-        <v>1492</v>
+        <v>1493</v>
       </c>
       <c r="D258" s="6" t="s">
         <v>29</v>
@@ -21655,19 +21670,19 @@
         <v>29</v>
       </c>
       <c r="H258" s="6" t="s">
-        <v>1493</v>
+        <v>1494</v>
       </c>
       <c r="I258" s="5" t="s">
         <v>29</v>
       </c>
       <c r="J258" s="6" t="s">
-        <v>1494</v>
+        <v>1495</v>
       </c>
       <c r="K258" s="6" t="s">
-        <v>1495</v>
+        <v>1496</v>
       </c>
       <c r="L258" s="6" t="s">
-        <v>1496</v>
+        <v>1497</v>
       </c>
       <c r="M258" s="5" t="s">
         <v>29</v>
@@ -21676,10 +21691,10 @@
         <v>29</v>
       </c>
       <c r="O258" s="6" t="s">
-        <v>1497</v>
+        <v>1498</v>
       </c>
       <c r="P258" s="6" t="s">
-        <v>1498</v>
+        <v>1499</v>
       </c>
       <c r="Q258" s="5" t="s">
         <v>29</v>
@@ -21699,10 +21714,10 @@
         <v>257</v>
       </c>
       <c r="B259" s="6" t="s">
-        <v>1499</v>
+        <v>1500</v>
       </c>
       <c r="C259" s="6" t="s">
-        <v>1500</v>
+        <v>1501</v>
       </c>
       <c r="D259" s="6" t="s">
         <v>29</v>
@@ -21717,7 +21732,7 @@
         <v>29</v>
       </c>
       <c r="H259" s="6" t="s">
-        <v>1501</v>
+        <v>1502</v>
       </c>
       <c r="I259" s="5" t="s">
         <v>29</v>
@@ -21726,10 +21741,10 @@
         <v>29</v>
       </c>
       <c r="K259" s="6" t="s">
-        <v>1502</v>
+        <v>1503</v>
       </c>
       <c r="L259" s="6" t="s">
-        <v>1503</v>
+        <v>1504</v>
       </c>
       <c r="M259" s="5" t="s">
         <v>29</v>
@@ -21741,7 +21756,7 @@
         <v>29</v>
       </c>
       <c r="P259" s="6" t="s">
-        <v>1504</v>
+        <v>1505</v>
       </c>
       <c r="Q259" s="5" t="s">
         <v>29</v>
@@ -21764,7 +21779,7 @@
         <v>957</v>
       </c>
       <c r="C260" s="7" t="s">
-        <v>1505</v>
+        <v>1506</v>
       </c>
       <c r="D260" s="7" t="s">
         <v>29</v>
@@ -21779,7 +21794,7 @@
         <v>29</v>
       </c>
       <c r="H260" s="7" t="s">
-        <v>1506</v>
+        <v>1507</v>
       </c>
       <c r="I260" s="5" t="s">
         <v>29</v>
@@ -21788,10 +21803,10 @@
         <v>29</v>
       </c>
       <c r="K260" s="7" t="s">
-        <v>1507</v>
+        <v>1508</v>
       </c>
       <c r="L260" s="7" t="s">
-        <v>1508</v>
+        <v>1509</v>
       </c>
       <c r="M260" s="5" t="s">
         <v>29</v>
@@ -21803,7 +21818,7 @@
         <v>29</v>
       </c>
       <c r="P260" s="7" t="s">
-        <v>1509</v>
+        <v>1510</v>
       </c>
       <c r="Q260" s="5" t="s">
         <v>29</v>
@@ -21826,7 +21841,7 @@
         <v>957</v>
       </c>
       <c r="C261" s="7" t="s">
-        <v>1510</v>
+        <v>1511</v>
       </c>
       <c r="D261" s="7" t="s">
         <v>29</v>
@@ -21865,7 +21880,7 @@
         <v>29</v>
       </c>
       <c r="P261" s="7" t="s">
-        <v>1511</v>
+        <v>1512</v>
       </c>
       <c r="Q261" s="5" t="s">
         <v>29</v>
@@ -21877,7 +21892,7 @@
         <v>29</v>
       </c>
       <c r="T261" s="7" t="s">
-        <v>1426</v>
+        <v>1428</v>
       </c>
     </row>
     <row r="262" spans="1:20">
@@ -21888,7 +21903,7 @@
         <v>957</v>
       </c>
       <c r="C262" s="7" t="s">
-        <v>1512</v>
+        <v>1513</v>
       </c>
       <c r="D262" s="7" t="s">
         <v>29</v>
@@ -21903,7 +21918,7 @@
         <v>29</v>
       </c>
       <c r="H262" s="7" t="s">
-        <v>1513</v>
+        <v>1514</v>
       </c>
       <c r="I262" s="5" t="s">
         <v>29</v>
@@ -21915,7 +21930,7 @@
         <v>29</v>
       </c>
       <c r="L262" s="7" t="s">
-        <v>1514</v>
+        <v>1515</v>
       </c>
       <c r="M262" s="5" t="s">
         <v>29</v>
@@ -21927,7 +21942,7 @@
         <v>29</v>
       </c>
       <c r="P262" s="7" t="s">
-        <v>1515</v>
+        <v>1516</v>
       </c>
       <c r="Q262" s="5" t="s">
         <v>29</v>
@@ -21950,7 +21965,7 @@
         <v>957</v>
       </c>
       <c r="C263" s="7" t="s">
-        <v>1516</v>
+        <v>1517</v>
       </c>
       <c r="D263" s="7" t="s">
         <v>29</v>
@@ -21965,7 +21980,7 @@
         <v>29</v>
       </c>
       <c r="H263" s="7" t="s">
-        <v>1517</v>
+        <v>1518</v>
       </c>
       <c r="I263" s="5" t="s">
         <v>29</v>
@@ -21974,7 +21989,7 @@
         <v>29</v>
       </c>
       <c r="K263" s="7" t="s">
-        <v>1518</v>
+        <v>1519</v>
       </c>
       <c r="L263" s="7" t="s">
         <v>29</v>
@@ -21989,7 +22004,7 @@
         <v>29</v>
       </c>
       <c r="P263" s="7" t="s">
-        <v>1519</v>
+        <v>1520</v>
       </c>
       <c r="Q263" s="5" t="s">
         <v>29</v>
@@ -22012,7 +22027,7 @@
         <v>957</v>
       </c>
       <c r="C264" s="7" t="s">
-        <v>1520</v>
+        <v>1521</v>
       </c>
       <c r="D264" s="7" t="s">
         <v>29</v>
@@ -22051,7 +22066,7 @@
         <v>29</v>
       </c>
       <c r="P264" s="7" t="s">
-        <v>29</v>
+        <v>1522</v>
       </c>
       <c r="Q264" s="5" t="s">
         <v>29</v>
@@ -22063,7 +22078,7 @@
         <v>29</v>
       </c>
       <c r="T264" s="7" t="s">
-        <v>1426</v>
+        <v>29</v>
       </c>
     </row>
     <row r="265" spans="1:20">
@@ -22074,7 +22089,7 @@
         <v>975</v>
       </c>
       <c r="C265" s="7" t="s">
-        <v>1521</v>
+        <v>1523</v>
       </c>
       <c r="D265" s="7" t="s">
         <v>29</v>
@@ -22089,37 +22104,37 @@
         <v>29</v>
       </c>
       <c r="H265" s="7" t="s">
-        <v>1522</v>
+        <v>1524</v>
       </c>
       <c r="I265" s="5" t="s">
         <v>29</v>
       </c>
       <c r="J265" s="7" t="s">
-        <v>1523</v>
+        <v>1525</v>
       </c>
       <c r="K265" s="7" t="s">
         <v>29</v>
       </c>
       <c r="L265" s="7" t="s">
-        <v>1524</v>
+        <v>1526</v>
       </c>
       <c r="M265" s="5" t="s">
         <v>29</v>
       </c>
       <c r="N265" s="7" t="s">
+        <v>1527</v>
+      </c>
+      <c r="O265" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P265" s="7" t="s">
+        <v>1528</v>
+      </c>
+      <c r="Q265" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="R265" s="7" t="s">
         <v>1525</v>
-      </c>
-      <c r="O265" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="P265" s="7" t="s">
-        <v>1526</v>
-      </c>
-      <c r="Q265" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="R265" s="7" t="s">
-        <v>1523</v>
       </c>
       <c r="S265" s="7" t="s">
         <v>29</v>
@@ -22136,7 +22151,7 @@
         <v>975</v>
       </c>
       <c r="C266" s="7" t="s">
-        <v>1527</v>
+        <v>1529</v>
       </c>
       <c r="D266" s="7" t="s">
         <v>29</v>
@@ -22151,7 +22166,7 @@
         <v>29</v>
       </c>
       <c r="H266" s="7" t="s">
-        <v>1528</v>
+        <v>1530</v>
       </c>
       <c r="I266" s="5" t="s">
         <v>29</v>
@@ -22160,10 +22175,10 @@
         <v>29</v>
       </c>
       <c r="K266" s="7" t="s">
-        <v>1529</v>
+        <v>1531</v>
       </c>
       <c r="L266" s="7" t="s">
-        <v>1530</v>
+        <v>1532</v>
       </c>
       <c r="M266" s="5" t="s">
         <v>29</v>
@@ -22172,10 +22187,10 @@
         <v>29</v>
       </c>
       <c r="O266" s="7" t="s">
-        <v>1529</v>
+        <v>1531</v>
       </c>
       <c r="P266" s="7" t="s">
-        <v>1531</v>
+        <v>1533</v>
       </c>
       <c r="Q266" s="5" t="s">
         <v>29</v>
@@ -22198,7 +22213,7 @@
         <v>1104</v>
       </c>
       <c r="C267" s="7" t="s">
-        <v>1532</v>
+        <v>1534</v>
       </c>
       <c r="D267" s="7" t="s">
         <v>29</v>
@@ -22260,7 +22275,7 @@
         <v>975</v>
       </c>
       <c r="C268" s="7" t="s">
-        <v>1533</v>
+        <v>1535</v>
       </c>
       <c r="D268" s="7" t="s">
         <v>29</v>
@@ -22287,7 +22302,7 @@
         <v>29</v>
       </c>
       <c r="L268" s="7" t="s">
-        <v>1534</v>
+        <v>1536</v>
       </c>
       <c r="M268" s="5" t="s">
         <v>29</v>
@@ -22296,10 +22311,10 @@
         <v>29</v>
       </c>
       <c r="O268" s="7" t="s">
-        <v>1535</v>
+        <v>1537</v>
       </c>
       <c r="P268" s="7" t="s">
-        <v>1536</v>
+        <v>1538</v>
       </c>
       <c r="Q268" s="5" t="s">
         <v>29</v>
@@ -22322,7 +22337,7 @@
         <v>975</v>
       </c>
       <c r="C269" s="7" t="s">
-        <v>1537</v>
+        <v>1539</v>
       </c>
       <c r="D269" s="7" t="s">
         <v>29</v>
@@ -22361,7 +22376,7 @@
         <v>29</v>
       </c>
       <c r="P269" s="7" t="s">
-        <v>1538</v>
+        <v>1540</v>
       </c>
       <c r="Q269" s="5" t="s">
         <v>29</v>
@@ -22384,7 +22399,7 @@
         <v>975</v>
       </c>
       <c r="C270" s="7" t="s">
-        <v>1539</v>
+        <v>1541</v>
       </c>
       <c r="D270" s="7" t="s">
         <v>29</v>
@@ -22399,7 +22414,7 @@
         <v>29</v>
       </c>
       <c r="H270" s="7" t="s">
-        <v>1540</v>
+        <v>1542</v>
       </c>
       <c r="I270" s="5" t="s">
         <v>29</v>
@@ -22411,7 +22426,7 @@
         <v>29</v>
       </c>
       <c r="L270" s="7" t="s">
-        <v>1541</v>
+        <v>1543</v>
       </c>
       <c r="M270" s="5" t="s">
         <v>29</v>
@@ -22423,7 +22438,7 @@
         <v>29</v>
       </c>
       <c r="P270" s="7" t="s">
-        <v>1542</v>
+        <v>1544</v>
       </c>
       <c r="Q270" s="5" t="s">
         <v>29</v>
@@ -22446,7 +22461,7 @@
         <v>975</v>
       </c>
       <c r="C271" s="7" t="s">
-        <v>1543</v>
+        <v>1545</v>
       </c>
       <c r="D271" s="7" t="s">
         <v>29</v>
@@ -22461,7 +22476,7 @@
         <v>29</v>
       </c>
       <c r="H271" s="7" t="s">
-        <v>1544</v>
+        <v>1546</v>
       </c>
       <c r="I271" s="5" t="s">
         <v>29</v>
@@ -22470,13 +22485,13 @@
         <v>29</v>
       </c>
       <c r="K271" s="7" t="s">
-        <v>1545</v>
+        <v>1547</v>
       </c>
       <c r="L271" s="7" t="s">
-        <v>1546</v>
+        <v>1548</v>
       </c>
       <c r="M271" s="7" t="s">
-        <v>1547</v>
+        <v>1549</v>
       </c>
       <c r="N271" s="7" t="s">
         <v>29</v>
@@ -22485,7 +22500,7 @@
         <v>29</v>
       </c>
       <c r="P271" s="7" t="s">
-        <v>1548</v>
+        <v>1550</v>
       </c>
       <c r="Q271" s="5" t="s">
         <v>29</v>
@@ -22508,7 +22523,7 @@
         <v>962</v>
       </c>
       <c r="C272" s="7" t="s">
-        <v>1549</v>
+        <v>1551</v>
       </c>
       <c r="D272" s="7" t="s">
         <v>29</v>
@@ -22523,7 +22538,7 @@
         <v>29</v>
       </c>
       <c r="H272" s="7" t="s">
-        <v>1550</v>
+        <v>1552</v>
       </c>
       <c r="I272" s="5" t="s">
         <v>29</v>
@@ -22535,7 +22550,7 @@
         <v>29</v>
       </c>
       <c r="L272" s="7" t="s">
-        <v>1551</v>
+        <v>1553</v>
       </c>
       <c r="M272" s="5" t="s">
         <v>29</v>
@@ -22547,7 +22562,7 @@
         <v>29</v>
       </c>
       <c r="P272" s="7" t="s">
-        <v>1552</v>
+        <v>1554</v>
       </c>
       <c r="Q272" s="5" t="s">
         <v>29</v>
@@ -22570,7 +22585,7 @@
         <v>962</v>
       </c>
       <c r="C273" s="7" t="s">
-        <v>1553</v>
+        <v>1555</v>
       </c>
       <c r="D273" s="7" t="s">
         <v>29</v>
@@ -22585,31 +22600,31 @@
         <v>29</v>
       </c>
       <c r="H273" s="7" t="s">
-        <v>1554</v>
+        <v>1556</v>
       </c>
       <c r="I273" s="5" t="s">
         <v>29</v>
       </c>
       <c r="J273" s="7" t="s">
-        <v>1555</v>
+        <v>1557</v>
       </c>
       <c r="K273" s="7" t="s">
-        <v>1556</v>
+        <v>1558</v>
       </c>
       <c r="L273" s="7" t="s">
-        <v>1557</v>
+        <v>1559</v>
       </c>
       <c r="M273" s="7" t="s">
         <v>1141</v>
       </c>
       <c r="N273" s="7" t="s">
-        <v>1558</v>
+        <v>1560</v>
       </c>
       <c r="O273" s="7" t="s">
         <v>29</v>
       </c>
       <c r="P273" s="7" t="s">
-        <v>1559</v>
+        <v>1561</v>
       </c>
       <c r="Q273" s="5" t="s">
         <v>29</v>
@@ -22632,7 +22647,7 @@
         <v>962</v>
       </c>
       <c r="C274" s="7" t="s">
-        <v>1560</v>
+        <v>1562</v>
       </c>
       <c r="D274" s="7" t="s">
         <v>29</v>
@@ -22647,7 +22662,7 @@
         <v>29</v>
       </c>
       <c r="H274" s="7" t="s">
-        <v>1561</v>
+        <v>1563</v>
       </c>
       <c r="I274" s="5" t="s">
         <v>29</v>
@@ -22659,7 +22674,7 @@
         <v>29</v>
       </c>
       <c r="L274" s="7" t="s">
-        <v>1562</v>
+        <v>1564</v>
       </c>
       <c r="M274" s="5" t="s">
         <v>29</v>
@@ -22671,7 +22686,7 @@
         <v>29</v>
       </c>
       <c r="P274" s="7" t="s">
-        <v>1563</v>
+        <v>1565</v>
       </c>
       <c r="Q274" s="5" t="s">
         <v>29</v>
@@ -22694,7 +22709,7 @@
         <v>962</v>
       </c>
       <c r="C275" s="7" t="s">
-        <v>1564</v>
+        <v>1566</v>
       </c>
       <c r="D275" s="7" t="s">
         <v>29</v>
@@ -22709,7 +22724,7 @@
         <v>29</v>
       </c>
       <c r="H275" s="7" t="s">
-        <v>1565</v>
+        <v>1567</v>
       </c>
       <c r="I275" s="5" t="s">
         <v>29</v>
@@ -22721,7 +22736,7 @@
         <v>29</v>
       </c>
       <c r="L275" s="7" t="s">
-        <v>1566</v>
+        <v>1568</v>
       </c>
       <c r="M275" s="5" t="s">
         <v>29</v>
@@ -22733,7 +22748,7 @@
         <v>29</v>
       </c>
       <c r="P275" s="7" t="s">
-        <v>1567</v>
+        <v>1569</v>
       </c>
       <c r="Q275" s="5" t="s">
         <v>29</v>
@@ -22756,7 +22771,7 @@
         <v>962</v>
       </c>
       <c r="C276" s="7" t="s">
-        <v>1568</v>
+        <v>1570</v>
       </c>
       <c r="D276" s="7" t="s">
         <v>29</v>
@@ -22771,31 +22786,31 @@
         <v>29</v>
       </c>
       <c r="H276" s="7" t="s">
-        <v>1569</v>
+        <v>1571</v>
       </c>
       <c r="I276" s="5" t="s">
         <v>29</v>
       </c>
       <c r="J276" s="7" t="s">
-        <v>1570</v>
+        <v>1572</v>
       </c>
       <c r="K276" s="7" t="s">
-        <v>1571</v>
+        <v>1573</v>
       </c>
       <c r="L276" s="7" t="s">
-        <v>1572</v>
+        <v>1574</v>
       </c>
       <c r="M276" s="5" t="s">
         <v>29</v>
       </c>
       <c r="N276" s="7" t="s">
-        <v>1573</v>
+        <v>1575</v>
       </c>
       <c r="O276" s="7" t="s">
-        <v>1574</v>
+        <v>1576</v>
       </c>
       <c r="P276" s="7" t="s">
-        <v>1575</v>
+        <v>1577</v>
       </c>
       <c r="Q276" s="5" t="s">
         <v>29</v>
@@ -22818,7 +22833,7 @@
         <v>975</v>
       </c>
       <c r="C277" s="7" t="s">
-        <v>1576</v>
+        <v>1578</v>
       </c>
       <c r="D277" s="7" t="s">
         <v>29</v>
@@ -22845,7 +22860,7 @@
         <v>29</v>
       </c>
       <c r="L277" s="7" t="s">
-        <v>1577</v>
+        <v>1579</v>
       </c>
       <c r="M277" s="5" t="s">
         <v>29</v>
@@ -22857,7 +22872,7 @@
         <v>29</v>
       </c>
       <c r="P277" s="7" t="s">
-        <v>1578</v>
+        <v>1580</v>
       </c>
       <c r="Q277" s="5" t="s">
         <v>29</v>
@@ -22880,7 +22895,7 @@
         <v>1050</v>
       </c>
       <c r="C278" s="7" t="s">
-        <v>1579</v>
+        <v>1581</v>
       </c>
       <c r="D278" s="7" t="s">
         <v>29</v>
@@ -22895,7 +22910,7 @@
         <v>29</v>
       </c>
       <c r="H278" s="7" t="s">
-        <v>1580</v>
+        <v>1582</v>
       </c>
       <c r="I278" s="5" t="s">
         <v>29</v>
@@ -22904,10 +22919,10 @@
         <v>29</v>
       </c>
       <c r="K278" s="7" t="s">
-        <v>1581</v>
+        <v>1583</v>
       </c>
       <c r="L278" s="7" t="s">
-        <v>1582</v>
+        <v>1584</v>
       </c>
       <c r="M278" s="5" t="s">
         <v>29</v>
@@ -22916,10 +22931,10 @@
         <v>29</v>
       </c>
       <c r="O278" s="7" t="s">
-        <v>1583</v>
+        <v>1585</v>
       </c>
       <c r="P278" s="7" t="s">
-        <v>1584</v>
+        <v>1586</v>
       </c>
       <c r="Q278" s="5" t="s">
         <v>29</v>
@@ -22942,7 +22957,7 @@
         <v>1050</v>
       </c>
       <c r="C279" s="7" t="s">
-        <v>1585</v>
+        <v>1587</v>
       </c>
       <c r="D279" s="7" t="s">
         <v>29</v>
@@ -22981,7 +22996,7 @@
         <v>29</v>
       </c>
       <c r="P279" s="7" t="s">
-        <v>1586</v>
+        <v>1588</v>
       </c>
       <c r="Q279" s="5" t="s">
         <v>29</v>
@@ -23004,7 +23019,7 @@
         <v>1104</v>
       </c>
       <c r="C280" s="7" t="s">
-        <v>1587</v>
+        <v>1589</v>
       </c>
       <c r="D280" s="7" t="s">
         <v>29</v>
@@ -23019,19 +23034,19 @@
         <v>29</v>
       </c>
       <c r="H280" s="7" t="s">
-        <v>1588</v>
+        <v>1590</v>
       </c>
       <c r="I280" s="5" t="s">
         <v>29</v>
       </c>
       <c r="J280" s="7" t="s">
-        <v>1589</v>
+        <v>1591</v>
       </c>
       <c r="K280" s="7" t="s">
-        <v>1590</v>
+        <v>1592</v>
       </c>
       <c r="L280" s="7" t="s">
-        <v>1591</v>
+        <v>1593</v>
       </c>
       <c r="M280" s="5" t="s">
         <v>29</v>
@@ -23040,10 +23055,10 @@
         <v>29</v>
       </c>
       <c r="O280" s="7" t="s">
-        <v>1592</v>
+        <v>1594</v>
       </c>
       <c r="P280" s="7" t="s">
-        <v>1593</v>
+        <v>1595</v>
       </c>
       <c r="Q280" s="5" t="s">
         <v>29</v>
@@ -23066,7 +23081,7 @@
         <v>1352</v>
       </c>
       <c r="C281" s="7" t="s">
-        <v>1594</v>
+        <v>1596</v>
       </c>
       <c r="D281" s="7" t="s">
         <v>29</v>
@@ -23081,19 +23096,19 @@
         <v>29</v>
       </c>
       <c r="H281" s="7" t="s">
-        <v>1595</v>
+        <v>1597</v>
       </c>
       <c r="I281" s="5" t="s">
         <v>29</v>
       </c>
       <c r="J281" s="7" t="s">
-        <v>1596</v>
+        <v>1598</v>
       </c>
       <c r="K281" s="7" t="s">
-        <v>1597</v>
+        <v>1599</v>
       </c>
       <c r="L281" s="7" t="s">
-        <v>1598</v>
+        <v>1600</v>
       </c>
       <c r="M281" s="5" t="s">
         <v>29</v>
@@ -23102,10 +23117,10 @@
         <v>29</v>
       </c>
       <c r="O281" s="7" t="s">
-        <v>1599</v>
+        <v>1601</v>
       </c>
       <c r="P281" s="7" t="s">
-        <v>1600</v>
+        <v>1602</v>
       </c>
       <c r="Q281" s="5" t="s">
         <v>29</v>
@@ -23128,7 +23143,7 @@
         <v>1072</v>
       </c>
       <c r="C282" s="7" t="s">
-        <v>1601</v>
+        <v>1603</v>
       </c>
       <c r="D282" s="7" t="s">
         <v>29</v>
@@ -23143,19 +23158,19 @@
         <v>29</v>
       </c>
       <c r="H282" s="7" t="s">
-        <v>1602</v>
+        <v>1604</v>
       </c>
       <c r="I282" s="7" t="s">
-        <v>1603</v>
+        <v>1605</v>
       </c>
       <c r="J282" s="7" t="s">
-        <v>1604</v>
+        <v>1606</v>
       </c>
       <c r="K282" s="7" t="s">
-        <v>1605</v>
+        <v>1607</v>
       </c>
       <c r="L282" s="7" t="s">
-        <v>1606</v>
+        <v>1608</v>
       </c>
       <c r="M282" s="5" t="s">
         <v>29</v>
@@ -23164,19 +23179,19 @@
         <v>29</v>
       </c>
       <c r="O282" s="7" t="s">
-        <v>1607</v>
+        <v>1609</v>
       </c>
       <c r="P282" s="7" t="s">
-        <v>29</v>
+        <v>1610</v>
       </c>
       <c r="Q282" s="5" t="s">
         <v>29</v>
       </c>
       <c r="R282" s="7" t="s">
-        <v>29</v>
+        <v>1611</v>
       </c>
       <c r="S282" s="7" t="s">
-        <v>29</v>
+        <v>1612</v>
       </c>
       <c r="T282" s="7" t="s">
         <v>29</v>
@@ -23190,7 +23205,7 @@
         <v>1072</v>
       </c>
       <c r="C283" s="7" t="s">
-        <v>1608</v>
+        <v>1613</v>
       </c>
       <c r="D283" s="7" t="s">
         <v>29</v>
@@ -23229,7 +23244,7 @@
         <v>29</v>
       </c>
       <c r="P283" s="7" t="s">
-        <v>1609</v>
+        <v>1614</v>
       </c>
       <c r="Q283" s="5" t="s">
         <v>29</v>
@@ -23249,10 +23264,10 @@
         <v>282</v>
       </c>
       <c r="B284" s="7" t="s">
-        <v>1479</v>
+        <v>1480</v>
       </c>
       <c r="C284" s="7" t="s">
-        <v>1610</v>
+        <v>1615</v>
       </c>
       <c r="D284" s="7" t="s">
         <v>29</v>
@@ -23267,7 +23282,7 @@
         <v>29</v>
       </c>
       <c r="H284" s="7" t="s">
-        <v>1611</v>
+        <v>1616</v>
       </c>
       <c r="I284" s="5" t="s">
         <v>29</v>
@@ -23279,19 +23294,19 @@
         <v>29</v>
       </c>
       <c r="L284" s="7" t="s">
-        <v>1612</v>
+        <v>1617</v>
       </c>
       <c r="M284" s="7" t="s">
         <v>1141</v>
       </c>
       <c r="N284" s="7" t="s">
-        <v>1613</v>
+        <v>1618</v>
       </c>
       <c r="O284" s="7" t="s">
         <v>29</v>
       </c>
       <c r="P284" s="7" t="s">
-        <v>1614</v>
+        <v>1619</v>
       </c>
       <c r="Q284" s="5" t="s">
         <v>29</v>
@@ -23314,7 +23329,7 @@
         <v>967</v>
       </c>
       <c r="C285" s="7" t="s">
-        <v>1615</v>
+        <v>1620</v>
       </c>
       <c r="D285" s="7" t="s">
         <v>29</v>
@@ -23329,19 +23344,19 @@
         <v>29</v>
       </c>
       <c r="H285" s="7" t="s">
-        <v>1616</v>
+        <v>1621</v>
       </c>
       <c r="I285" s="5" t="s">
         <v>29</v>
       </c>
       <c r="J285" s="7" t="s">
-        <v>1617</v>
+        <v>1622</v>
       </c>
       <c r="K285" s="7" t="s">
-        <v>1618</v>
+        <v>1623</v>
       </c>
       <c r="L285" s="7" t="s">
-        <v>1619</v>
+        <v>1624</v>
       </c>
       <c r="M285" s="5" t="s">
         <v>29</v>
@@ -23350,10 +23365,10 @@
         <v>29</v>
       </c>
       <c r="O285" s="7" t="s">
-        <v>1620</v>
+        <v>1625</v>
       </c>
       <c r="P285" s="7" t="s">
-        <v>1621</v>
+        <v>1626</v>
       </c>
       <c r="Q285" s="5" t="s">
         <v>29</v>
@@ -23376,7 +23391,7 @@
         <v>1072</v>
       </c>
       <c r="C286" s="7" t="s">
-        <v>1622</v>
+        <v>1627</v>
       </c>
       <c r="D286" s="7" t="s">
         <v>29</v>
@@ -23391,19 +23406,19 @@
         <v>29</v>
       </c>
       <c r="H286" s="7" t="s">
-        <v>1623</v>
+        <v>1628</v>
       </c>
       <c r="I286" s="7" t="s">
-        <v>1624</v>
+        <v>1629</v>
       </c>
       <c r="J286" s="7" t="s">
-        <v>1625</v>
+        <v>1630</v>
       </c>
       <c r="K286" s="7" t="s">
-        <v>1626</v>
+        <v>1631</v>
       </c>
       <c r="L286" s="7" t="s">
-        <v>1627</v>
+        <v>1632</v>
       </c>
       <c r="M286" s="5" t="s">
         <v>29</v>
@@ -23415,7 +23430,7 @@
         <v>29</v>
       </c>
       <c r="P286" s="7" t="s">
-        <v>1628</v>
+        <v>1633</v>
       </c>
       <c r="Q286" s="5" t="s">
         <v>29</v>
@@ -23438,7 +23453,7 @@
         <v>975</v>
       </c>
       <c r="C287" s="7" t="s">
-        <v>1629</v>
+        <v>1634</v>
       </c>
       <c r="D287" s="7" t="s">
         <v>29</v>
@@ -23453,31 +23468,31 @@
         <v>29</v>
       </c>
       <c r="H287" s="7" t="s">
-        <v>1630</v>
+        <v>1635</v>
       </c>
       <c r="I287" s="5" t="s">
         <v>29</v>
       </c>
       <c r="J287" s="7" t="s">
-        <v>1631</v>
+        <v>1636</v>
       </c>
       <c r="K287" s="7" t="s">
         <v>29</v>
       </c>
       <c r="L287" s="7" t="s">
-        <v>1632</v>
+        <v>1637</v>
       </c>
       <c r="M287" s="5" t="s">
         <v>29</v>
       </c>
       <c r="N287" s="7" t="s">
-        <v>1631</v>
+        <v>1636</v>
       </c>
       <c r="O287" s="7" t="s">
         <v>29</v>
       </c>
       <c r="P287" s="7" t="s">
-        <v>1633</v>
+        <v>1638</v>
       </c>
       <c r="Q287" s="5" t="s">
         <v>29</v>
@@ -24130,66 +24145,68 @@
     <hyperlink ref="P262" r:id="rId631"/>
     <hyperlink ref="H263" r:id="rId632"/>
     <hyperlink ref="P263" r:id="rId633"/>
-    <hyperlink ref="H265" r:id="rId634"/>
-    <hyperlink ref="L265" r:id="rId635"/>
-    <hyperlink ref="P265" r:id="rId636"/>
-    <hyperlink ref="H266" r:id="rId637"/>
-    <hyperlink ref="L266" r:id="rId638"/>
-    <hyperlink ref="P266" r:id="rId639"/>
-    <hyperlink ref="L268" r:id="rId640"/>
-    <hyperlink ref="P268" r:id="rId641"/>
-    <hyperlink ref="P269" r:id="rId642"/>
-    <hyperlink ref="H270" r:id="rId643"/>
-    <hyperlink ref="L270" r:id="rId644"/>
-    <hyperlink ref="P270" r:id="rId645"/>
-    <hyperlink ref="H271" r:id="rId646"/>
-    <hyperlink ref="L271" r:id="rId647"/>
-    <hyperlink ref="P271" r:id="rId648"/>
-    <hyperlink ref="H272" r:id="rId649"/>
-    <hyperlink ref="L272" r:id="rId650"/>
-    <hyperlink ref="P272" r:id="rId651"/>
-    <hyperlink ref="H273" r:id="rId652"/>
-    <hyperlink ref="L273" r:id="rId653"/>
-    <hyperlink ref="P273" r:id="rId654"/>
-    <hyperlink ref="H274" r:id="rId655"/>
-    <hyperlink ref="L274" r:id="rId656"/>
-    <hyperlink ref="P274" r:id="rId657"/>
-    <hyperlink ref="H275" r:id="rId658"/>
-    <hyperlink ref="L275" r:id="rId659"/>
-    <hyperlink ref="P275" r:id="rId660"/>
-    <hyperlink ref="H276" r:id="rId661"/>
-    <hyperlink ref="L276" r:id="rId662"/>
-    <hyperlink ref="P276" r:id="rId663"/>
-    <hyperlink ref="L277" r:id="rId664"/>
-    <hyperlink ref="P277" r:id="rId665"/>
-    <hyperlink ref="H278" r:id="rId666"/>
-    <hyperlink ref="L278" r:id="rId667"/>
-    <hyperlink ref="P278" r:id="rId668"/>
-    <hyperlink ref="P279" r:id="rId669"/>
-    <hyperlink ref="H280" r:id="rId670"/>
-    <hyperlink ref="L280" r:id="rId671"/>
-    <hyperlink ref="P280" r:id="rId672"/>
-    <hyperlink ref="H281" r:id="rId673"/>
-    <hyperlink ref="L281" r:id="rId674"/>
-    <hyperlink ref="P281" r:id="rId675"/>
-    <hyperlink ref="H282" r:id="rId676"/>
-    <hyperlink ref="L282" r:id="rId677"/>
-    <hyperlink ref="P283" r:id="rId678"/>
-    <hyperlink ref="H284" r:id="rId679"/>
-    <hyperlink ref="L284" r:id="rId680"/>
-    <hyperlink ref="P284" r:id="rId681"/>
-    <hyperlink ref="H285" r:id="rId682"/>
-    <hyperlink ref="L285" r:id="rId683"/>
-    <hyperlink ref="P285" r:id="rId684"/>
-    <hyperlink ref="H286" r:id="rId685"/>
-    <hyperlink ref="L286" r:id="rId686"/>
-    <hyperlink ref="P286" r:id="rId687"/>
-    <hyperlink ref="H287" r:id="rId688"/>
-    <hyperlink ref="L287" r:id="rId689"/>
-    <hyperlink ref="P287" r:id="rId690"/>
+    <hyperlink ref="P264" r:id="rId634"/>
+    <hyperlink ref="H265" r:id="rId635"/>
+    <hyperlink ref="L265" r:id="rId636"/>
+    <hyperlink ref="P265" r:id="rId637"/>
+    <hyperlink ref="H266" r:id="rId638"/>
+    <hyperlink ref="L266" r:id="rId639"/>
+    <hyperlink ref="P266" r:id="rId640"/>
+    <hyperlink ref="L268" r:id="rId641"/>
+    <hyperlink ref="P268" r:id="rId642"/>
+    <hyperlink ref="P269" r:id="rId643"/>
+    <hyperlink ref="H270" r:id="rId644"/>
+    <hyperlink ref="L270" r:id="rId645"/>
+    <hyperlink ref="P270" r:id="rId646"/>
+    <hyperlink ref="H271" r:id="rId647"/>
+    <hyperlink ref="L271" r:id="rId648"/>
+    <hyperlink ref="P271" r:id="rId649"/>
+    <hyperlink ref="H272" r:id="rId650"/>
+    <hyperlink ref="L272" r:id="rId651"/>
+    <hyperlink ref="P272" r:id="rId652"/>
+    <hyperlink ref="H273" r:id="rId653"/>
+    <hyperlink ref="L273" r:id="rId654"/>
+    <hyperlink ref="P273" r:id="rId655"/>
+    <hyperlink ref="H274" r:id="rId656"/>
+    <hyperlink ref="L274" r:id="rId657"/>
+    <hyperlink ref="P274" r:id="rId658"/>
+    <hyperlink ref="H275" r:id="rId659"/>
+    <hyperlink ref="L275" r:id="rId660"/>
+    <hyperlink ref="P275" r:id="rId661"/>
+    <hyperlink ref="H276" r:id="rId662"/>
+    <hyperlink ref="L276" r:id="rId663"/>
+    <hyperlink ref="P276" r:id="rId664"/>
+    <hyperlink ref="L277" r:id="rId665"/>
+    <hyperlink ref="P277" r:id="rId666"/>
+    <hyperlink ref="H278" r:id="rId667"/>
+    <hyperlink ref="L278" r:id="rId668"/>
+    <hyperlink ref="P278" r:id="rId669"/>
+    <hyperlink ref="P279" r:id="rId670"/>
+    <hyperlink ref="H280" r:id="rId671"/>
+    <hyperlink ref="L280" r:id="rId672"/>
+    <hyperlink ref="P280" r:id="rId673"/>
+    <hyperlink ref="H281" r:id="rId674"/>
+    <hyperlink ref="L281" r:id="rId675"/>
+    <hyperlink ref="P281" r:id="rId676"/>
+    <hyperlink ref="H282" r:id="rId677"/>
+    <hyperlink ref="L282" r:id="rId678"/>
+    <hyperlink ref="P282" r:id="rId679"/>
+    <hyperlink ref="P283" r:id="rId680"/>
+    <hyperlink ref="H284" r:id="rId681"/>
+    <hyperlink ref="L284" r:id="rId682"/>
+    <hyperlink ref="P284" r:id="rId683"/>
+    <hyperlink ref="H285" r:id="rId684"/>
+    <hyperlink ref="L285" r:id="rId685"/>
+    <hyperlink ref="P285" r:id="rId686"/>
+    <hyperlink ref="H286" r:id="rId687"/>
+    <hyperlink ref="L286" r:id="rId688"/>
+    <hyperlink ref="P286" r:id="rId689"/>
+    <hyperlink ref="H287" r:id="rId690"/>
+    <hyperlink ref="L287" r:id="rId691"/>
+    <hyperlink ref="P287" r:id="rId692"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId691"/>
+  <drawing r:id="rId693"/>
 </worksheet>
 </file>
 
@@ -24218,7 +24235,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>1642</v>
+        <v>1647</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -24525,7 +24542,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>1643</v>
+        <v>1648</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -24835,7 +24852,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>1644</v>
+        <v>1649</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -24985,7 +25002,7 @@
         <v>1352</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>1594</v>
+        <v>1596</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>29</v>
@@ -25000,19 +25017,19 @@
         <v>29</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>1595</v>
+        <v>1597</v>
       </c>
       <c r="I4" s="5" t="s">
         <v>29</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>1596</v>
+        <v>1598</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>1597</v>
+        <v>1599</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>1598</v>
+        <v>1600</v>
       </c>
       <c r="M4" s="5" t="s">
         <v>29</v>
@@ -25021,10 +25038,10 @@
         <v>29</v>
       </c>
       <c r="O4" s="7" t="s">
-        <v>1599</v>
+        <v>1601</v>
       </c>
       <c r="P4" s="7" t="s">
-        <v>1600</v>
+        <v>1602</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>29</v>
@@ -25080,7 +25097,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>1645</v>
+        <v>1650</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -28863,7 +28880,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>1646</v>
+        <v>1651</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -29043,7 +29060,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>1647</v>
+        <v>1652</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -29286,7 +29303,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>1648</v>
+        <v>1653</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -29994,7 +30011,7 @@
         <v>962</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>1428</v>
+        <v>1429</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>29</v>
@@ -30009,19 +30026,19 @@
         <v>29</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>1429</v>
+        <v>1430</v>
       </c>
       <c r="I13" s="5" t="s">
         <v>29</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>1430</v>
+        <v>1431</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>1431</v>
+        <v>1432</v>
       </c>
       <c r="L13" s="6" t="s">
-        <v>1432</v>
+        <v>1433</v>
       </c>
       <c r="M13" s="5" t="s">
         <v>29</v>
@@ -30030,10 +30047,10 @@
         <v>29</v>
       </c>
       <c r="O13" s="6" t="s">
-        <v>1433</v>
+        <v>1434</v>
       </c>
       <c r="P13" s="6" t="s">
-        <v>1434</v>
+        <v>1435</v>
       </c>
       <c r="Q13" s="6" t="s">
         <v>1141</v>
@@ -30056,7 +30073,7 @@
         <v>962</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>1549</v>
+        <v>1551</v>
       </c>
       <c r="D14" s="7" t="s">
         <v>29</v>
@@ -30071,7 +30088,7 @@
         <v>29</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>1550</v>
+        <v>1552</v>
       </c>
       <c r="I14" s="5" t="s">
         <v>29</v>
@@ -30083,7 +30100,7 @@
         <v>29</v>
       </c>
       <c r="L14" s="7" t="s">
-        <v>1551</v>
+        <v>1553</v>
       </c>
       <c r="M14" s="5" t="s">
         <v>29</v>
@@ -30095,7 +30112,7 @@
         <v>29</v>
       </c>
       <c r="P14" s="7" t="s">
-        <v>1552</v>
+        <v>1554</v>
       </c>
       <c r="Q14" s="5" t="s">
         <v>29</v>
@@ -30118,7 +30135,7 @@
         <v>962</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>1553</v>
+        <v>1555</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>29</v>
@@ -30133,31 +30150,31 @@
         <v>29</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>1554</v>
+        <v>1556</v>
       </c>
       <c r="I15" s="5" t="s">
         <v>29</v>
       </c>
       <c r="J15" s="7" t="s">
-        <v>1555</v>
+        <v>1557</v>
       </c>
       <c r="K15" s="7" t="s">
-        <v>1556</v>
+        <v>1558</v>
       </c>
       <c r="L15" s="7" t="s">
-        <v>1557</v>
+        <v>1559</v>
       </c>
       <c r="M15" s="7" t="s">
         <v>1141</v>
       </c>
       <c r="N15" s="7" t="s">
-        <v>1558</v>
+        <v>1560</v>
       </c>
       <c r="O15" s="7" t="s">
         <v>29</v>
       </c>
       <c r="P15" s="7" t="s">
-        <v>1559</v>
+        <v>1561</v>
       </c>
       <c r="Q15" s="5" t="s">
         <v>29</v>
@@ -30180,7 +30197,7 @@
         <v>962</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>1560</v>
+        <v>1562</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>29</v>
@@ -30195,7 +30212,7 @@
         <v>29</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>1561</v>
+        <v>1563</v>
       </c>
       <c r="I16" s="5" t="s">
         <v>29</v>
@@ -30207,7 +30224,7 @@
         <v>29</v>
       </c>
       <c r="L16" s="7" t="s">
-        <v>1562</v>
+        <v>1564</v>
       </c>
       <c r="M16" s="5" t="s">
         <v>29</v>
@@ -30219,7 +30236,7 @@
         <v>29</v>
       </c>
       <c r="P16" s="7" t="s">
-        <v>1563</v>
+        <v>1565</v>
       </c>
       <c r="Q16" s="5" t="s">
         <v>29</v>
@@ -30242,7 +30259,7 @@
         <v>962</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>1564</v>
+        <v>1566</v>
       </c>
       <c r="D17" s="7" t="s">
         <v>29</v>
@@ -30257,7 +30274,7 @@
         <v>29</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>1565</v>
+        <v>1567</v>
       </c>
       <c r="I17" s="5" t="s">
         <v>29</v>
@@ -30269,7 +30286,7 @@
         <v>29</v>
       </c>
       <c r="L17" s="7" t="s">
-        <v>1566</v>
+        <v>1568</v>
       </c>
       <c r="M17" s="5" t="s">
         <v>29</v>
@@ -30281,7 +30298,7 @@
         <v>29</v>
       </c>
       <c r="P17" s="7" t="s">
-        <v>1567</v>
+        <v>1569</v>
       </c>
       <c r="Q17" s="5" t="s">
         <v>29</v>
@@ -30304,7 +30321,7 @@
         <v>962</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>1568</v>
+        <v>1570</v>
       </c>
       <c r="D18" s="7" t="s">
         <v>29</v>
@@ -30319,31 +30336,31 @@
         <v>29</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>1569</v>
+        <v>1571</v>
       </c>
       <c r="I18" s="5" t="s">
         <v>29</v>
       </c>
       <c r="J18" s="7" t="s">
-        <v>1570</v>
+        <v>1572</v>
       </c>
       <c r="K18" s="7" t="s">
-        <v>1571</v>
+        <v>1573</v>
       </c>
       <c r="L18" s="7" t="s">
-        <v>1572</v>
+        <v>1574</v>
       </c>
       <c r="M18" s="5" t="s">
         <v>29</v>
       </c>
       <c r="N18" s="7" t="s">
-        <v>1573</v>
+        <v>1575</v>
       </c>
       <c r="O18" s="7" t="s">
-        <v>1574</v>
+        <v>1576</v>
       </c>
       <c r="P18" s="7" t="s">
-        <v>1575</v>
+        <v>1577</v>
       </c>
       <c r="Q18" s="5" t="s">
         <v>29</v>
@@ -30437,7 +30454,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>1649</v>
+        <v>1654</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -30617,7 +30634,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>1650</v>
+        <v>1655</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -30797,7 +30814,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>1651</v>
+        <v>1656</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -30882,10 +30899,10 @@
         <v>1</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>1479</v>
+        <v>1480</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>1480</v>
+        <v>1481</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>29</v>
@@ -30900,19 +30917,19 @@
         <v>29</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>1481</v>
+        <v>1482</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>1482</v>
+        <v>1483</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>1483</v>
+        <v>1484</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>1484</v>
+        <v>1485</v>
       </c>
       <c r="L3" s="6" t="s">
-        <v>1485</v>
+        <v>1486</v>
       </c>
       <c r="M3" s="5" t="s">
         <v>29</v>
@@ -30924,7 +30941,7 @@
         <v>29</v>
       </c>
       <c r="P3" s="6" t="s">
-        <v>1486</v>
+        <v>1487</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>29</v>
@@ -30944,10 +30961,10 @@
         <v>2</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>1479</v>
+        <v>1480</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>1610</v>
+        <v>1615</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>29</v>
@@ -30962,7 +30979,7 @@
         <v>29</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>1611</v>
+        <v>1616</v>
       </c>
       <c r="I4" s="5" t="s">
         <v>29</v>
@@ -30974,19 +30991,19 @@
         <v>29</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>1612</v>
+        <v>1617</v>
       </c>
       <c r="M4" s="7" t="s">
         <v>1141</v>
       </c>
       <c r="N4" s="7" t="s">
-        <v>1613</v>
+        <v>1618</v>
       </c>
       <c r="O4" s="7" t="s">
         <v>29</v>
       </c>
       <c r="P4" s="7" t="s">
-        <v>1614</v>
+        <v>1619</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>29</v>
@@ -31042,7 +31059,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>1634</v>
+        <v>1639</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -31750,7 +31767,7 @@
         <v>957</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>1505</v>
+        <v>1506</v>
       </c>
       <c r="D13" s="7" t="s">
         <v>29</v>
@@ -31765,7 +31782,7 @@
         <v>29</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>1506</v>
+        <v>1507</v>
       </c>
       <c r="I13" s="5" t="s">
         <v>29</v>
@@ -31774,10 +31791,10 @@
         <v>29</v>
       </c>
       <c r="K13" s="7" t="s">
-        <v>1507</v>
+        <v>1508</v>
       </c>
       <c r="L13" s="7" t="s">
-        <v>1508</v>
+        <v>1509</v>
       </c>
       <c r="M13" s="5" t="s">
         <v>29</v>
@@ -31789,7 +31806,7 @@
         <v>29</v>
       </c>
       <c r="P13" s="7" t="s">
-        <v>1509</v>
+        <v>1510</v>
       </c>
       <c r="Q13" s="5" t="s">
         <v>29</v>
@@ -31812,7 +31829,7 @@
         <v>957</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>1510</v>
+        <v>1511</v>
       </c>
       <c r="D14" s="7" t="s">
         <v>29</v>
@@ -31851,7 +31868,7 @@
         <v>29</v>
       </c>
       <c r="P14" s="7" t="s">
-        <v>1511</v>
+        <v>1512</v>
       </c>
       <c r="Q14" s="5" t="s">
         <v>29</v>
@@ -31863,7 +31880,7 @@
         <v>29</v>
       </c>
       <c r="T14" s="7" t="s">
-        <v>1426</v>
+        <v>1428</v>
       </c>
     </row>
     <row r="15" spans="1:20">
@@ -31874,7 +31891,7 @@
         <v>957</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>1512</v>
+        <v>1513</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>29</v>
@@ -31889,7 +31906,7 @@
         <v>29</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>1513</v>
+        <v>1514</v>
       </c>
       <c r="I15" s="5" t="s">
         <v>29</v>
@@ -31901,7 +31918,7 @@
         <v>29</v>
       </c>
       <c r="L15" s="7" t="s">
-        <v>1514</v>
+        <v>1515</v>
       </c>
       <c r="M15" s="5" t="s">
         <v>29</v>
@@ -31913,7 +31930,7 @@
         <v>29</v>
       </c>
       <c r="P15" s="7" t="s">
-        <v>1515</v>
+        <v>1516</v>
       </c>
       <c r="Q15" s="5" t="s">
         <v>29</v>
@@ -31936,7 +31953,7 @@
         <v>957</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>1516</v>
+        <v>1517</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>29</v>
@@ -31951,7 +31968,7 @@
         <v>29</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>1517</v>
+        <v>1518</v>
       </c>
       <c r="I16" s="5" t="s">
         <v>29</v>
@@ -31960,7 +31977,7 @@
         <v>29</v>
       </c>
       <c r="K16" s="7" t="s">
-        <v>1518</v>
+        <v>1519</v>
       </c>
       <c r="L16" s="7" t="s">
         <v>29</v>
@@ -31975,7 +31992,7 @@
         <v>29</v>
       </c>
       <c r="P16" s="7" t="s">
-        <v>1519</v>
+        <v>1520</v>
       </c>
       <c r="Q16" s="5" t="s">
         <v>29</v>
@@ -31998,7 +32015,7 @@
         <v>957</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>1520</v>
+        <v>1521</v>
       </c>
       <c r="D17" s="7" t="s">
         <v>29</v>
@@ -32037,7 +32054,7 @@
         <v>29</v>
       </c>
       <c r="P17" s="7" t="s">
-        <v>29</v>
+        <v>1522</v>
       </c>
       <c r="Q17" s="5" t="s">
         <v>29</v>
@@ -32049,7 +32066,7 @@
         <v>29</v>
       </c>
       <c r="T17" s="7" t="s">
-        <v>1426</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -32090,6 +32107,7 @@
     <hyperlink ref="P15" r:id="rId31"/>
     <hyperlink ref="H16" r:id="rId32"/>
     <hyperlink ref="P16" r:id="rId33"/>
+    <hyperlink ref="P17" r:id="rId34"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -32120,7 +32138,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>1652</v>
+        <v>1657</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -32270,7 +32288,7 @@
         <v>1104</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>1532</v>
+        <v>1534</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>29</v>
@@ -32332,7 +32350,7 @@
         <v>1104</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>1587</v>
+        <v>1589</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>29</v>
@@ -32347,19 +32365,19 @@
         <v>29</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>1588</v>
+        <v>1590</v>
       </c>
       <c r="I5" s="5" t="s">
         <v>29</v>
       </c>
       <c r="J5" s="7" t="s">
-        <v>1589</v>
+        <v>1591</v>
       </c>
       <c r="K5" s="7" t="s">
-        <v>1590</v>
+        <v>1592</v>
       </c>
       <c r="L5" s="7" t="s">
-        <v>1591</v>
+        <v>1593</v>
       </c>
       <c r="M5" s="5" t="s">
         <v>29</v>
@@ -32368,10 +32386,10 @@
         <v>29</v>
       </c>
       <c r="O5" s="7" t="s">
-        <v>1592</v>
+        <v>1594</v>
       </c>
       <c r="P5" s="7" t="s">
-        <v>1593</v>
+        <v>1595</v>
       </c>
       <c r="Q5" s="5" t="s">
         <v>29</v>
@@ -32425,7 +32443,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>1653</v>
+        <v>1658</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -32605,7 +32623,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>1654</v>
+        <v>1659</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -33174,7 +33192,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>1655</v>
+        <v>1660</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -33510,7 +33528,7 @@
         <v>967</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>1615</v>
+        <v>1620</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>29</v>
@@ -33525,19 +33543,19 @@
         <v>29</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>1616</v>
+        <v>1621</v>
       </c>
       <c r="I7" s="5" t="s">
         <v>29</v>
       </c>
       <c r="J7" s="7" t="s">
-        <v>1617</v>
+        <v>1622</v>
       </c>
       <c r="K7" s="7" t="s">
-        <v>1618</v>
+        <v>1623</v>
       </c>
       <c r="L7" s="7" t="s">
-        <v>1619</v>
+        <v>1624</v>
       </c>
       <c r="M7" s="5" t="s">
         <v>29</v>
@@ -33546,10 +33564,10 @@
         <v>29</v>
       </c>
       <c r="O7" s="7" t="s">
-        <v>1620</v>
+        <v>1625</v>
       </c>
       <c r="P7" s="7" t="s">
-        <v>1621</v>
+        <v>1626</v>
       </c>
       <c r="Q7" s="5" t="s">
         <v>29</v>
@@ -33613,7 +33631,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>1656</v>
+        <v>1661</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -33791,7 +33809,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>1657</v>
+        <v>1662</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -34035,7 +34053,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>1658</v>
+        <v>1663</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -34120,10 +34138,10 @@
         <v>1</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>1470</v>
+        <v>1471</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>1471</v>
+        <v>1472</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>29</v>
@@ -34162,7 +34180,7 @@
         <v>29</v>
       </c>
       <c r="P3" s="6" t="s">
-        <v>1472</v>
+        <v>1473</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>29</v>
@@ -34213,7 +34231,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>1659</v>
+        <v>1664</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -34298,10 +34316,10 @@
         <v>1</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>1473</v>
+        <v>1474</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>1474</v>
+        <v>1475</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>29</v>
@@ -34316,7 +34334,7 @@
         <v>29</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>1475</v>
+        <v>1476</v>
       </c>
       <c r="I3" s="5" t="s">
         <v>29</v>
@@ -34325,10 +34343,10 @@
         <v>29</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>1476</v>
+        <v>1477</v>
       </c>
       <c r="L3" s="6" t="s">
-        <v>1477</v>
+        <v>1478</v>
       </c>
       <c r="M3" s="5" t="s">
         <v>29</v>
@@ -34340,7 +34358,7 @@
         <v>29</v>
       </c>
       <c r="P3" s="6" t="s">
-        <v>1478</v>
+        <v>1479</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>29</v>
@@ -34393,7 +34411,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>1660</v>
+        <v>1665</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -37212,7 +37230,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>1661</v>
+        <v>1666</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -37362,7 +37380,7 @@
         <v>1150</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>1450</v>
+        <v>1451</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>29</v>
@@ -37377,7 +37395,7 @@
         <v>29</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>1451</v>
+        <v>1452</v>
       </c>
       <c r="I4" s="5" t="s">
         <v>29</v>
@@ -37389,19 +37407,19 @@
         <v>29</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>1452</v>
+        <v>1453</v>
       </c>
       <c r="M4" s="5" t="s">
         <v>29</v>
       </c>
       <c r="N4" s="6" t="s">
-        <v>1453</v>
+        <v>1454</v>
       </c>
       <c r="O4" s="6" t="s">
         <v>29</v>
       </c>
       <c r="P4" s="6" t="s">
-        <v>1454</v>
+        <v>1455</v>
       </c>
       <c r="Q4" s="5" t="s">
         <v>29</v>
@@ -37457,7 +37475,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>1635</v>
+        <v>1640</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -37637,7 +37655,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>1662</v>
+        <v>1667</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -37962,7 +37980,7 @@
         <v>29</v>
       </c>
       <c r="T6" s="6" t="s">
-        <v>1426</v>
+        <v>1428</v>
       </c>
     </row>
     <row r="7" spans="1:20">
@@ -37973,7 +37991,7 @@
         <v>1127</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>1435</v>
+        <v>1436</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>29</v>
@@ -37988,31 +38006,31 @@
         <v>29</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>1436</v>
+        <v>1437</v>
       </c>
       <c r="I7" s="5" t="s">
         <v>29</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>1437</v>
+        <v>1438</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>1438</v>
+        <v>1439</v>
       </c>
       <c r="L7" s="6" t="s">
-        <v>1439</v>
+        <v>1440</v>
       </c>
       <c r="M7" s="6" t="s">
-        <v>1440</v>
+        <v>1441</v>
       </c>
       <c r="N7" s="6" t="s">
         <v>29</v>
       </c>
       <c r="O7" s="6" t="s">
-        <v>1441</v>
+        <v>1442</v>
       </c>
       <c r="P7" s="6" t="s">
-        <v>1442</v>
+        <v>1443</v>
       </c>
       <c r="Q7" s="5" t="s">
         <v>29</v>
@@ -38035,7 +38053,7 @@
         <v>1127</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>1463</v>
+        <v>1464</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>29</v>
@@ -38050,19 +38068,19 @@
         <v>29</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>1464</v>
+        <v>1465</v>
       </c>
       <c r="I8" s="5" t="s">
         <v>29</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>1465</v>
+        <v>1466</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>1466</v>
+        <v>1467</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>1467</v>
+        <v>1468</v>
       </c>
       <c r="M8" s="5" t="s">
         <v>29</v>
@@ -38071,10 +38089,10 @@
         <v>29</v>
       </c>
       <c r="O8" s="6" t="s">
-        <v>1468</v>
+        <v>1469</v>
       </c>
       <c r="P8" s="6" t="s">
-        <v>1469</v>
+        <v>1470</v>
       </c>
       <c r="Q8" s="5" t="s">
         <v>29</v>
@@ -38097,7 +38115,7 @@
         <v>1127</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>1487</v>
+        <v>1488</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>29</v>
@@ -38112,7 +38130,7 @@
         <v>29</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>1488</v>
+        <v>1489</v>
       </c>
       <c r="I9" s="5" t="s">
         <v>29</v>
@@ -38124,10 +38142,10 @@
         <v>29</v>
       </c>
       <c r="L9" s="6" t="s">
-        <v>1489</v>
+        <v>1490</v>
       </c>
       <c r="M9" s="6" t="s">
-        <v>1490</v>
+        <v>1491</v>
       </c>
       <c r="N9" s="6" t="s">
         <v>29</v>
@@ -38136,7 +38154,7 @@
         <v>29</v>
       </c>
       <c r="P9" s="6" t="s">
-        <v>1491</v>
+        <v>1492</v>
       </c>
       <c r="Q9" s="5" t="s">
         <v>29</v>
@@ -38159,7 +38177,7 @@
         <v>1127</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>1492</v>
+        <v>1493</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>29</v>
@@ -38174,19 +38192,19 @@
         <v>29</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>1493</v>
+        <v>1494</v>
       </c>
       <c r="I10" s="5" t="s">
         <v>29</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>1494</v>
+        <v>1495</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>1495</v>
+        <v>1496</v>
       </c>
       <c r="L10" s="6" t="s">
-        <v>1496</v>
+        <v>1497</v>
       </c>
       <c r="M10" s="5" t="s">
         <v>29</v>
@@ -38195,10 +38213,10 @@
         <v>29</v>
       </c>
       <c r="O10" s="6" t="s">
-        <v>1497</v>
+        <v>1498</v>
       </c>
       <c r="P10" s="6" t="s">
-        <v>1498</v>
+        <v>1499</v>
       </c>
       <c r="Q10" s="5" t="s">
         <v>29</v>
@@ -38268,7 +38286,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>1663</v>
+        <v>1668</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -38353,10 +38371,10 @@
         <v>1</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>1499</v>
+        <v>1500</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>1500</v>
+        <v>1501</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>29</v>
@@ -38371,7 +38389,7 @@
         <v>29</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>1501</v>
+        <v>1502</v>
       </c>
       <c r="I3" s="5" t="s">
         <v>29</v>
@@ -38380,10 +38398,10 @@
         <v>29</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>1502</v>
+        <v>1503</v>
       </c>
       <c r="L3" s="6" t="s">
-        <v>1503</v>
+        <v>1504</v>
       </c>
       <c r="M3" s="5" t="s">
         <v>29</v>
@@ -38395,7 +38413,7 @@
         <v>29</v>
       </c>
       <c r="P3" s="6" t="s">
-        <v>1504</v>
+        <v>1505</v>
       </c>
       <c r="Q3" s="5" t="s">
         <v>29</v>
@@ -38448,7 +38466,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>1664</v>
+        <v>1669</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -40490,7 +40508,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>1636</v>
+        <v>1641</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -40670,7 +40688,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>1637</v>
+        <v>1642</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -42370,7 +42388,7 @@
         <v>975</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>1521</v>
+        <v>1523</v>
       </c>
       <c r="D29" s="7" t="s">
         <v>29</v>
@@ -42385,37 +42403,37 @@
         <v>29</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>1522</v>
+        <v>1524</v>
       </c>
       <c r="I29" s="5" t="s">
         <v>29</v>
       </c>
       <c r="J29" s="7" t="s">
-        <v>1523</v>
+        <v>1525</v>
       </c>
       <c r="K29" s="7" t="s">
         <v>29</v>
       </c>
       <c r="L29" s="7" t="s">
-        <v>1524</v>
+        <v>1526</v>
       </c>
       <c r="M29" s="5" t="s">
         <v>29</v>
       </c>
       <c r="N29" s="7" t="s">
+        <v>1527</v>
+      </c>
+      <c r="O29" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="P29" s="7" t="s">
+        <v>1528</v>
+      </c>
+      <c r="Q29" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="R29" s="7" t="s">
         <v>1525</v>
-      </c>
-      <c r="O29" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="P29" s="7" t="s">
-        <v>1526</v>
-      </c>
-      <c r="Q29" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="R29" s="7" t="s">
-        <v>1523</v>
       </c>
       <c r="S29" s="7" t="s">
         <v>29</v>
@@ -42432,7 +42450,7 @@
         <v>975</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>1527</v>
+        <v>1529</v>
       </c>
       <c r="D30" s="7" t="s">
         <v>29</v>
@@ -42447,7 +42465,7 @@
         <v>29</v>
       </c>
       <c r="H30" s="7" t="s">
-        <v>1528</v>
+        <v>1530</v>
       </c>
       <c r="I30" s="5" t="s">
         <v>29</v>
@@ -42456,10 +42474,10 @@
         <v>29</v>
       </c>
       <c r="K30" s="7" t="s">
-        <v>1529</v>
+        <v>1531</v>
       </c>
       <c r="L30" s="7" t="s">
-        <v>1530</v>
+        <v>1532</v>
       </c>
       <c r="M30" s="5" t="s">
         <v>29</v>
@@ -42468,10 +42486,10 @@
         <v>29</v>
       </c>
       <c r="O30" s="7" t="s">
-        <v>1529</v>
+        <v>1531</v>
       </c>
       <c r="P30" s="7" t="s">
-        <v>1531</v>
+        <v>1533</v>
       </c>
       <c r="Q30" s="5" t="s">
         <v>29</v>
@@ -42494,7 +42512,7 @@
         <v>975</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>1533</v>
+        <v>1535</v>
       </c>
       <c r="D31" s="7" t="s">
         <v>29</v>
@@ -42521,7 +42539,7 @@
         <v>29</v>
       </c>
       <c r="L31" s="7" t="s">
-        <v>1534</v>
+        <v>1536</v>
       </c>
       <c r="M31" s="5" t="s">
         <v>29</v>
@@ -42530,10 +42548,10 @@
         <v>29</v>
       </c>
       <c r="O31" s="7" t="s">
-        <v>1535</v>
+        <v>1537</v>
       </c>
       <c r="P31" s="7" t="s">
-        <v>1536</v>
+        <v>1538</v>
       </c>
       <c r="Q31" s="5" t="s">
         <v>29</v>
@@ -42556,7 +42574,7 @@
         <v>975</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>1537</v>
+        <v>1539</v>
       </c>
       <c r="D32" s="7" t="s">
         <v>29</v>
@@ -42595,7 +42613,7 @@
         <v>29</v>
       </c>
       <c r="P32" s="7" t="s">
-        <v>1538</v>
+        <v>1540</v>
       </c>
       <c r="Q32" s="5" t="s">
         <v>29</v>
@@ -42618,7 +42636,7 @@
         <v>975</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>1539</v>
+        <v>1541</v>
       </c>
       <c r="D33" s="7" t="s">
         <v>29</v>
@@ -42633,7 +42651,7 @@
         <v>29</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>1540</v>
+        <v>1542</v>
       </c>
       <c r="I33" s="5" t="s">
         <v>29</v>
@@ -42645,7 +42663,7 @@
         <v>29</v>
       </c>
       <c r="L33" s="7" t="s">
-        <v>1541</v>
+        <v>1543</v>
       </c>
       <c r="M33" s="5" t="s">
         <v>29</v>
@@ -42657,7 +42675,7 @@
         <v>29</v>
       </c>
       <c r="P33" s="7" t="s">
-        <v>1542</v>
+        <v>1544</v>
       </c>
       <c r="Q33" s="5" t="s">
         <v>29</v>
@@ -42680,7 +42698,7 @@
         <v>975</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>1543</v>
+        <v>1545</v>
       </c>
       <c r="D34" s="7" t="s">
         <v>29</v>
@@ -42695,7 +42713,7 @@
         <v>29</v>
       </c>
       <c r="H34" s="7" t="s">
-        <v>1544</v>
+        <v>1546</v>
       </c>
       <c r="I34" s="5" t="s">
         <v>29</v>
@@ -42704,13 +42722,13 @@
         <v>29</v>
       </c>
       <c r="K34" s="7" t="s">
-        <v>1545</v>
+        <v>1547</v>
       </c>
       <c r="L34" s="7" t="s">
-        <v>1546</v>
+        <v>1548</v>
       </c>
       <c r="M34" s="7" t="s">
-        <v>1547</v>
+        <v>1549</v>
       </c>
       <c r="N34" s="7" t="s">
         <v>29</v>
@@ -42719,7 +42737,7 @@
         <v>29</v>
       </c>
       <c r="P34" s="7" t="s">
-        <v>1548</v>
+        <v>1550</v>
       </c>
       <c r="Q34" s="5" t="s">
         <v>29</v>
@@ -42742,7 +42760,7 @@
         <v>975</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>1576</v>
+        <v>1578</v>
       </c>
       <c r="D35" s="7" t="s">
         <v>29</v>
@@ -42769,7 +42787,7 @@
         <v>29</v>
       </c>
       <c r="L35" s="7" t="s">
-        <v>1577</v>
+        <v>1579</v>
       </c>
       <c r="M35" s="5" t="s">
         <v>29</v>
@@ -42781,7 +42799,7 @@
         <v>29</v>
       </c>
       <c r="P35" s="7" t="s">
-        <v>1578</v>
+        <v>1580</v>
       </c>
       <c r="Q35" s="5" t="s">
         <v>29</v>
@@ -42804,7 +42822,7 @@
         <v>975</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>1629</v>
+        <v>1634</v>
       </c>
       <c r="D36" s="7" t="s">
         <v>29</v>
@@ -42819,31 +42837,31 @@
         <v>29</v>
       </c>
       <c r="H36" s="7" t="s">
-        <v>1630</v>
+        <v>1635</v>
       </c>
       <c r="I36" s="5" t="s">
         <v>29</v>
       </c>
       <c r="J36" s="7" t="s">
-        <v>1631</v>
+        <v>1636</v>
       </c>
       <c r="K36" s="7" t="s">
         <v>29</v>
       </c>
       <c r="L36" s="7" t="s">
-        <v>1632</v>
+        <v>1637</v>
       </c>
       <c r="M36" s="5" t="s">
         <v>29</v>
       </c>
       <c r="N36" s="7" t="s">
-        <v>1631</v>
+        <v>1636</v>
       </c>
       <c r="O36" s="7" t="s">
         <v>29</v>
       </c>
       <c r="P36" s="7" t="s">
-        <v>1633</v>
+        <v>1638</v>
       </c>
       <c r="Q36" s="5" t="s">
         <v>29</v>
@@ -42983,7 +43001,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>1638</v>
+        <v>1643</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -44892,7 +44910,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>1639</v>
+        <v>1644</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -45166,7 +45184,7 @@
         <v>1072</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>1443</v>
+        <v>1444</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>29</v>
@@ -45181,19 +45199,19 @@
         <v>29</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>1444</v>
+        <v>1445</v>
       </c>
       <c r="I6" s="5" t="s">
         <v>29</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>1445</v>
+        <v>1446</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>1446</v>
+        <v>1447</v>
       </c>
       <c r="L6" s="6" t="s">
-        <v>1447</v>
+        <v>1448</v>
       </c>
       <c r="M6" s="5" t="s">
         <v>29</v>
@@ -45202,10 +45220,10 @@
         <v>29</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>1448</v>
+        <v>1449</v>
       </c>
       <c r="P6" s="6" t="s">
-        <v>1449</v>
+        <v>1450</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>29</v>
@@ -45228,7 +45246,7 @@
         <v>1072</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>1455</v>
+        <v>1456</v>
       </c>
       <c r="D7" s="6" t="s">
         <v>29</v>
@@ -45243,31 +45261,31 @@
         <v>29</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>1456</v>
+        <v>1457</v>
       </c>
       <c r="I7" s="5" t="s">
         <v>29</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>1457</v>
+        <v>1458</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>1458</v>
+        <v>1459</v>
       </c>
       <c r="L7" s="6" t="s">
-        <v>1459</v>
+        <v>1460</v>
       </c>
       <c r="M7" s="5" t="s">
         <v>29</v>
       </c>
       <c r="N7" s="6" t="s">
-        <v>1460</v>
+        <v>1461</v>
       </c>
       <c r="O7" s="6" t="s">
-        <v>1461</v>
+        <v>1462</v>
       </c>
       <c r="P7" s="6" t="s">
-        <v>1462</v>
+        <v>1463</v>
       </c>
       <c r="Q7" s="5" t="s">
         <v>29</v>
@@ -45290,7 +45308,7 @@
         <v>1072</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>1601</v>
+        <v>1603</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>29</v>
@@ -45305,19 +45323,19 @@
         <v>29</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>1602</v>
+        <v>1604</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>1603</v>
+        <v>1605</v>
       </c>
       <c r="J8" s="7" t="s">
-        <v>1604</v>
+        <v>1606</v>
       </c>
       <c r="K8" s="7" t="s">
-        <v>1605</v>
+        <v>1607</v>
       </c>
       <c r="L8" s="7" t="s">
-        <v>1606</v>
+        <v>1608</v>
       </c>
       <c r="M8" s="5" t="s">
         <v>29</v>
@@ -45326,19 +45344,19 @@
         <v>29</v>
       </c>
       <c r="O8" s="7" t="s">
-        <v>1607</v>
+        <v>1609</v>
       </c>
       <c r="P8" s="7" t="s">
-        <v>29</v>
+        <v>1610</v>
       </c>
       <c r="Q8" s="5" t="s">
         <v>29</v>
       </c>
       <c r="R8" s="7" t="s">
-        <v>29</v>
+        <v>1611</v>
       </c>
       <c r="S8" s="7" t="s">
-        <v>29</v>
+        <v>1612</v>
       </c>
       <c r="T8" s="7" t="s">
         <v>29</v>
@@ -45352,7 +45370,7 @@
         <v>1072</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>1608</v>
+        <v>1613</v>
       </c>
       <c r="D9" s="7" t="s">
         <v>29</v>
@@ -45391,7 +45409,7 @@
         <v>29</v>
       </c>
       <c r="P9" s="7" t="s">
-        <v>1609</v>
+        <v>1614</v>
       </c>
       <c r="Q9" s="5" t="s">
         <v>29</v>
@@ -45414,7 +45432,7 @@
         <v>1072</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>1622</v>
+        <v>1627</v>
       </c>
       <c r="D10" s="7" t="s">
         <v>29</v>
@@ -45429,19 +45447,19 @@
         <v>29</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>1623</v>
+        <v>1628</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>1624</v>
+        <v>1629</v>
       </c>
       <c r="J10" s="7" t="s">
-        <v>1625</v>
+        <v>1630</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>1626</v>
+        <v>1631</v>
       </c>
       <c r="L10" s="7" t="s">
-        <v>1627</v>
+        <v>1632</v>
       </c>
       <c r="M10" s="5" t="s">
         <v>29</v>
@@ -45453,7 +45471,7 @@
         <v>29</v>
       </c>
       <c r="P10" s="7" t="s">
-        <v>1628</v>
+        <v>1633</v>
       </c>
       <c r="Q10" s="5" t="s">
         <v>29</v>
@@ -45488,10 +45506,11 @@
     <hyperlink ref="P7" r:id="rId13"/>
     <hyperlink ref="H8" r:id="rId14"/>
     <hyperlink ref="L8" r:id="rId15"/>
-    <hyperlink ref="P9" r:id="rId16"/>
-    <hyperlink ref="H10" r:id="rId17"/>
-    <hyperlink ref="L10" r:id="rId18"/>
-    <hyperlink ref="P10" r:id="rId19"/>
+    <hyperlink ref="P8" r:id="rId16"/>
+    <hyperlink ref="P9" r:id="rId17"/>
+    <hyperlink ref="H10" r:id="rId18"/>
+    <hyperlink ref="L10" r:id="rId19"/>
+    <hyperlink ref="P10" r:id="rId20"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -45522,7 +45541,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>1640</v>
+        <v>1645</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -45796,7 +45815,7 @@
         <v>1050</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>1579</v>
+        <v>1581</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>29</v>
@@ -45811,7 +45830,7 @@
         <v>29</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>1580</v>
+        <v>1582</v>
       </c>
       <c r="I6" s="5" t="s">
         <v>29</v>
@@ -45820,10 +45839,10 @@
         <v>29</v>
       </c>
       <c r="K6" s="7" t="s">
-        <v>1581</v>
+        <v>1583</v>
       </c>
       <c r="L6" s="7" t="s">
-        <v>1582</v>
+        <v>1584</v>
       </c>
       <c r="M6" s="5" t="s">
         <v>29</v>
@@ -45832,10 +45851,10 @@
         <v>29</v>
       </c>
       <c r="O6" s="7" t="s">
-        <v>1583</v>
+        <v>1585</v>
       </c>
       <c r="P6" s="7" t="s">
-        <v>1584</v>
+        <v>1586</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>29</v>
@@ -45858,7 +45877,7 @@
         <v>1050</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>1585</v>
+        <v>1587</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>29</v>
@@ -45897,7 +45916,7 @@
         <v>29</v>
       </c>
       <c r="P7" s="7" t="s">
-        <v>1586</v>
+        <v>1588</v>
       </c>
       <c r="Q7" s="5" t="s">
         <v>29</v>
@@ -45958,7 +45977,7 @@
   <sheetData>
     <row r="1" spans="1:20">
       <c r="A1" s="1" t="s">
-        <v>1641</v>
+        <v>1646</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>

</xml_diff>